<commit_message>
self tanglegrams, per-segment RPM
</commit_message>
<xml_diff>
--- a/analyses/trees/RNA2/RNA2_Seq_IDs.xlsx
+++ b/analyses/trees/RNA2/RNA2_Seq_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/diverse_collections/github/analyses/trees/RNA2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdstengl/Google_Drive/Projects/Galbut_virus/Diverse_Collections/DiverseCollections/analyses/trees/RNA2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8959359-85E7-7A4D-BBF0-2DBFA6926AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D2F76C-C4E6-3140-B316-6D11EDD5D9FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33800" yWindow="500" windowWidth="26840" windowHeight="15940" xr2:uid="{1ABCC1F6-95A5-2146-8F8C-226ACC8CFFC1}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19500" xr2:uid="{1ABCC1F6-95A5-2146-8F8C-226ACC8CFFC1}"/>
   </bookViews>
   <sheets>
     <sheet name="RNA2_Seq_IDs" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="295">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="294">
   <si>
     <t>isolate</t>
   </si>
@@ -557,9 +557,6 @@
   </si>
   <si>
     <t>PQ625037</t>
-  </si>
-  <si>
-    <t>Unknown</t>
   </si>
   <si>
     <t>D_mel_USA_2023_Peach-9-F8_Galbut_virus_RNA2_Complete_CDS</t>
@@ -1768,7 +1765,7 @@
   <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="1" max="1" width="29" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -3224,7 +3221,7 @@
         <v>178</v>
       </c>
       <c r="C86" t="s">
-        <v>179</v>
+        <v>7</v>
       </c>
       <c r="D86">
         <v>2023</v>
@@ -3235,13 +3232,13 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
+        <v>179</v>
+      </c>
+      <c r="B87" t="s">
         <v>180</v>
       </c>
-      <c r="B87" t="s">
-        <v>181</v>
-      </c>
       <c r="C87" t="s">
-        <v>179</v>
+        <v>7</v>
       </c>
       <c r="D87">
         <v>2023</v>
@@ -3252,13 +3249,13 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
+        <v>181</v>
+      </c>
+      <c r="B88" t="s">
         <v>182</v>
       </c>
-      <c r="B88" t="s">
-        <v>183</v>
-      </c>
       <c r="C88" t="s">
-        <v>179</v>
+        <v>7</v>
       </c>
       <c r="D88">
         <v>2023</v>
@@ -3269,13 +3266,13 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
+        <v>183</v>
+      </c>
+      <c r="B89" t="s">
         <v>184</v>
       </c>
-      <c r="B89" t="s">
-        <v>185</v>
-      </c>
       <c r="C89" t="s">
-        <v>179</v>
+        <v>7</v>
       </c>
       <c r="D89">
         <v>2023</v>
@@ -3286,13 +3283,13 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
+        <v>185</v>
+      </c>
+      <c r="B90" t="s">
         <v>186</v>
       </c>
-      <c r="B90" t="s">
+      <c r="C90" t="s">
         <v>187</v>
-      </c>
-      <c r="C90" t="s">
-        <v>188</v>
       </c>
       <c r="D90">
         <v>2023</v>
@@ -3303,13 +3300,13 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
+        <v>188</v>
+      </c>
+      <c r="B91" t="s">
         <v>189</v>
       </c>
-      <c r="B91" t="s">
-        <v>190</v>
-      </c>
       <c r="C91" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D91">
         <v>2023</v>
@@ -3320,13 +3317,13 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
+        <v>190</v>
+      </c>
+      <c r="B92" t="s">
         <v>191</v>
       </c>
-      <c r="B92" t="s">
-        <v>192</v>
-      </c>
       <c r="C92" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D92">
         <v>2023</v>
@@ -3337,13 +3334,13 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
+        <v>192</v>
+      </c>
+      <c r="B93" t="s">
         <v>193</v>
       </c>
-      <c r="B93" t="s">
-        <v>194</v>
-      </c>
       <c r="C93" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D93">
         <v>2023</v>
@@ -3354,13 +3351,13 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
+        <v>194</v>
+      </c>
+      <c r="B94" t="s">
         <v>195</v>
       </c>
-      <c r="B94" t="s">
-        <v>196</v>
-      </c>
       <c r="C94" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D94">
         <v>2023</v>
@@ -3371,13 +3368,13 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
+        <v>196</v>
+      </c>
+      <c r="B95" t="s">
         <v>197</v>
       </c>
-      <c r="B95" t="s">
-        <v>198</v>
-      </c>
       <c r="C95" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D95">
         <v>2023</v>
@@ -3388,13 +3385,13 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
+        <v>198</v>
+      </c>
+      <c r="B96" t="s">
         <v>199</v>
       </c>
-      <c r="B96" t="s">
-        <v>200</v>
-      </c>
       <c r="C96" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D96">
         <v>2023</v>
@@ -3405,13 +3402,13 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
+        <v>200</v>
+      </c>
+      <c r="B97" t="s">
         <v>201</v>
       </c>
-      <c r="B97" t="s">
-        <v>202</v>
-      </c>
       <c r="C97" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D97">
         <v>2023</v>
@@ -3422,13 +3419,13 @@
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
+        <v>202</v>
+      </c>
+      <c r="B98" t="s">
         <v>203</v>
       </c>
-      <c r="B98" t="s">
-        <v>204</v>
-      </c>
       <c r="C98" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D98">
         <v>2023</v>
@@ -3439,13 +3436,13 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
+        <v>204</v>
+      </c>
+      <c r="B99" t="s">
         <v>205</v>
       </c>
-      <c r="B99" t="s">
-        <v>206</v>
-      </c>
       <c r="C99" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D99">
         <v>2023</v>
@@ -3456,13 +3453,13 @@
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
+        <v>206</v>
+      </c>
+      <c r="B100" t="s">
         <v>207</v>
       </c>
-      <c r="B100" t="s">
-        <v>208</v>
-      </c>
       <c r="C100" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D100">
         <v>2023</v>
@@ -3473,13 +3470,13 @@
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
+        <v>208</v>
+      </c>
+      <c r="B101" t="s">
         <v>209</v>
       </c>
-      <c r="B101" t="s">
-        <v>210</v>
-      </c>
       <c r="C101" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D101">
         <v>2023</v>
@@ -3490,13 +3487,13 @@
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
+        <v>210</v>
+      </c>
+      <c r="B102" t="s">
         <v>211</v>
       </c>
-      <c r="B102" t="s">
-        <v>212</v>
-      </c>
       <c r="C102" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D102">
         <v>2023</v>
@@ -3507,13 +3504,13 @@
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
+        <v>212</v>
+      </c>
+      <c r="B103" t="s">
         <v>213</v>
       </c>
-      <c r="B103" t="s">
-        <v>214</v>
-      </c>
       <c r="C103" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D103">
         <v>2023</v>
@@ -3524,13 +3521,13 @@
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
+        <v>214</v>
+      </c>
+      <c r="B104" t="s">
         <v>215</v>
       </c>
-      <c r="B104" t="s">
-        <v>216</v>
-      </c>
       <c r="C104" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D104">
         <v>2023</v>
@@ -3541,10 +3538,10 @@
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
+        <v>216</v>
+      </c>
+      <c r="B105" t="s">
         <v>217</v>
-      </c>
-      <c r="B105" t="s">
-        <v>218</v>
       </c>
       <c r="C105" t="s">
         <v>133</v>
@@ -3553,15 +3550,15 @@
         <v>2023</v>
       </c>
       <c r="E105" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
+        <v>219</v>
+      </c>
+      <c r="C106" t="s">
         <v>220</v>
-      </c>
-      <c r="C106" t="s">
-        <v>221</v>
       </c>
       <c r="D106">
         <v>2008</v>
@@ -3572,10 +3569,10 @@
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C107" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D107">
         <v>2008</v>
@@ -3586,10 +3583,10 @@
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C108" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D108">
         <v>2008</v>
@@ -3600,10 +3597,10 @@
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C109" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D109">
         <v>2008</v>
@@ -3614,10 +3611,10 @@
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C110" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D110">
         <v>2008</v>
@@ -3628,10 +3625,10 @@
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C111" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D111">
         <v>2008</v>
@@ -3642,7 +3639,7 @@
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C112" t="s">
         <v>7</v>
@@ -3656,7 +3653,7 @@
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B113" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C113" t="s">
         <v>7</v>
@@ -3670,7 +3667,7 @@
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B114" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C114" t="s">
         <v>7</v>
@@ -3684,7 +3681,7 @@
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B115" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C115" t="s">
         <v>7</v>
@@ -3698,7 +3695,7 @@
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B116" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C116" t="s">
         <v>7</v>
@@ -3712,7 +3709,7 @@
     </row>
     <row r="117" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B117" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C117" t="s">
         <v>7</v>
@@ -3726,7 +3723,7 @@
     </row>
     <row r="118" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B118" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C118" t="s">
         <v>7</v>
@@ -3740,7 +3737,7 @@
     </row>
     <row r="119" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B119" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C119" t="s">
         <v>7</v>
@@ -3754,7 +3751,7 @@
     </row>
     <row r="120" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B120" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C120" t="s">
         <v>7</v>
@@ -3768,7 +3765,7 @@
     </row>
     <row r="121" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B121" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C121" t="s">
         <v>7</v>
@@ -3782,7 +3779,7 @@
     </row>
     <row r="122" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B122" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C122" t="s">
         <v>7</v>
@@ -3796,7 +3793,7 @@
     </row>
     <row r="123" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B123" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C123" t="s">
         <v>7</v>
@@ -3810,7 +3807,7 @@
     </row>
     <row r="124" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B124" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C124" t="s">
         <v>7</v>
@@ -3824,7 +3821,7 @@
     </row>
     <row r="125" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B125" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C125" t="s">
         <v>7</v>
@@ -3838,7 +3835,7 @@
     </row>
     <row r="126" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B126" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C126" t="s">
         <v>7</v>
@@ -3852,7 +3849,7 @@
     </row>
     <row r="127" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B127" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C127" t="s">
         <v>7</v>
@@ -3866,7 +3863,7 @@
     </row>
     <row r="128" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B128" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C128" t="s">
         <v>7</v>
@@ -3880,7 +3877,7 @@
     </row>
     <row r="129" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B129" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C129" t="s">
         <v>7</v>
@@ -3894,7 +3891,7 @@
     </row>
     <row r="130" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B130" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C130" t="s">
         <v>7</v>
@@ -3908,7 +3905,7 @@
     </row>
     <row r="131" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B131" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C131" t="s">
         <v>7</v>
@@ -3922,7 +3919,7 @@
     </row>
     <row r="132" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B132" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C132" t="s">
         <v>7</v>
@@ -3936,7 +3933,7 @@
     </row>
     <row r="133" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B133" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C133" t="s">
         <v>7</v>
@@ -3950,7 +3947,7 @@
     </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B134" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C134" t="s">
         <v>7</v>
@@ -3964,7 +3961,7 @@
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B135" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C135" t="s">
         <v>7</v>
@@ -3978,7 +3975,7 @@
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B136" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C136" t="s">
         <v>7</v>
@@ -3992,7 +3989,7 @@
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B137" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C137" t="s">
         <v>7</v>
@@ -4006,7 +4003,7 @@
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B138" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C138" t="s">
         <v>7</v>
@@ -4020,7 +4017,7 @@
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B139" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C139" t="s">
         <v>7</v>
@@ -4034,7 +4031,7 @@
     </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B140" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C140" t="s">
         <v>7</v>
@@ -4048,7 +4045,7 @@
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B141" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="C141" t="s">
         <v>7</v>
@@ -4062,10 +4059,10 @@
     </row>
     <row r="142" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B142" t="s">
+        <v>256</v>
+      </c>
+      <c r="C142" t="s">
         <v>257</v>
-      </c>
-      <c r="C142" t="s">
-        <v>258</v>
       </c>
       <c r="D142">
         <v>1908</v>
@@ -4076,10 +4073,10 @@
     </row>
     <row r="143" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B143" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C143" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D143">
         <v>1930</v>
@@ -4090,10 +4087,10 @@
     </row>
     <row r="144" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B144" t="s">
+        <v>259</v>
+      </c>
+      <c r="C144" t="s">
         <v>260</v>
-      </c>
-      <c r="C144" t="s">
-        <v>261</v>
       </c>
       <c r="D144">
         <v>1919</v>
@@ -4104,10 +4101,10 @@
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B145" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C145" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D145">
         <v>1963</v>
@@ -4118,268 +4115,268 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B146" t="s">
+        <v>262</v>
+      </c>
+      <c r="C146" t="s">
         <v>263</v>
-      </c>
-      <c r="C146" t="s">
-        <v>264</v>
       </c>
       <c r="D146">
         <v>2000</v>
       </c>
       <c r="E146" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B147" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C147" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D147">
         <v>2011</v>
       </c>
       <c r="E147" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="B148" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C148" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D148">
         <v>2018</v>
       </c>
       <c r="E148" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B149" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C149" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D149">
         <v>2018</v>
       </c>
       <c r="E149" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B150" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C150" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D150">
         <v>2018</v>
       </c>
       <c r="E150" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B151" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C151" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D151">
         <v>2018</v>
       </c>
       <c r="E151" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B152" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C152" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D152">
         <v>2018</v>
       </c>
       <c r="E152" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B153" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C153" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D153">
         <v>2018</v>
       </c>
       <c r="E153" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B154" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C154" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D154">
         <v>2018</v>
       </c>
       <c r="E154" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B155" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C155" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D155">
         <v>2018</v>
       </c>
       <c r="E155" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="B156" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C156" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D156">
         <v>2018</v>
       </c>
       <c r="E156" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B157" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C157" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D157">
         <v>2018</v>
       </c>
       <c r="E157" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B158" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C158" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D158">
         <v>2018</v>
       </c>
       <c r="E158" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B159" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C159" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D159">
         <v>2018</v>
       </c>
       <c r="E159" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B160" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="C160" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D160">
         <v>2018</v>
       </c>
       <c r="E160" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B161" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C161" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D161">
         <v>2018</v>
       </c>
       <c r="E161" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reset seq ID files
</commit_message>
<xml_diff>
--- a/analyses/trees/RNA2/RNA2_Seq_IDs.xlsx
+++ b/analyses/trees/RNA2/RNA2_Seq_IDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mdstengl/Google_Drive/Projects/Galbut_virus/Diverse_Collections/DiverseCollections/analyses/trees/RNA2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lexikeene/Documents/Research/diverse_collections/github/analyses/trees/RNA2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0D2F76C-C4E6-3140-B316-6D11EDD5D9FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADBBA742-EAC2-6F46-80AC-D5478073657E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19500" xr2:uid="{1ABCC1F6-95A5-2146-8F8C-226ACC8CFFC1}"/>
+    <workbookView xWindow="33800" yWindow="500" windowWidth="26840" windowHeight="21100" xr2:uid="{1ABCC1F6-95A5-2146-8F8C-226ACC8CFFC1}"/>
   </bookViews>
   <sheets>
     <sheet name="RNA2_Seq_IDs" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="603" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="395">
   <si>
     <t>isolate</t>
   </si>
@@ -902,6 +902,309 @@
   </si>
   <si>
     <t>PV185893</t>
+  </si>
+  <si>
+    <t>sample_id</t>
+  </si>
+  <si>
+    <t>mel-20-TD-3</t>
+  </si>
+  <si>
+    <t>sim-20-TD-4</t>
+  </si>
+  <si>
+    <t>mel-21-MDS-9</t>
+  </si>
+  <si>
+    <t>500-F-11</t>
+  </si>
+  <si>
+    <t>500-F-41</t>
+  </si>
+  <si>
+    <t>500-F-67</t>
+  </si>
+  <si>
+    <t>500-M-16</t>
+  </si>
+  <si>
+    <t>500-M-17</t>
+  </si>
+  <si>
+    <t>500-M-54</t>
+  </si>
+  <si>
+    <t>500-M-57</t>
+  </si>
+  <si>
+    <t>500-M-60</t>
+  </si>
+  <si>
+    <t>500-M-61-2</t>
+  </si>
+  <si>
+    <t>500-M-61</t>
+  </si>
+  <si>
+    <t>500-M-65-2</t>
+  </si>
+  <si>
+    <t>500-M-65</t>
+  </si>
+  <si>
+    <t>500-M-71-2</t>
+  </si>
+  <si>
+    <t>500-M-83</t>
+  </si>
+  <si>
+    <t>500-M-84</t>
+  </si>
+  <si>
+    <t>500-M-F10</t>
+  </si>
+  <si>
+    <t>500-M-F11</t>
+  </si>
+  <si>
+    <t>500-M-G2</t>
+  </si>
+  <si>
+    <t>1020-A7</t>
+  </si>
+  <si>
+    <t>1020-B6</t>
+  </si>
+  <si>
+    <t>1020-C2</t>
+  </si>
+  <si>
+    <t>1020-D1</t>
+  </si>
+  <si>
+    <t>1020-D3</t>
+  </si>
+  <si>
+    <t>1020-F1</t>
+  </si>
+  <si>
+    <t>1020-F6</t>
+  </si>
+  <si>
+    <t>1020-F-31</t>
+  </si>
+  <si>
+    <t>1020-F-36</t>
+  </si>
+  <si>
+    <t>1020-F-40</t>
+  </si>
+  <si>
+    <t>1020-F-44</t>
+  </si>
+  <si>
+    <t>1020-F-0818-D4</t>
+  </si>
+  <si>
+    <t>1020-F-0818-D11</t>
+  </si>
+  <si>
+    <t>1020-G3</t>
+  </si>
+  <si>
+    <t>1020-M-8</t>
+  </si>
+  <si>
+    <t>1020-M-19</t>
+  </si>
+  <si>
+    <t>1020-M-0818-A5</t>
+  </si>
+  <si>
+    <t>1020-M-0818-A7</t>
+  </si>
+  <si>
+    <t>1020-M-0818-A10</t>
+  </si>
+  <si>
+    <t>1428-F-8</t>
+  </si>
+  <si>
+    <t>1428-F-21</t>
+  </si>
+  <si>
+    <t>1428-M-3</t>
+  </si>
+  <si>
+    <t>1428-M-4</t>
+  </si>
+  <si>
+    <t>1428-M-21</t>
+  </si>
+  <si>
+    <t>1428-M-42</t>
+  </si>
+  <si>
+    <t>Adobe-B4</t>
+  </si>
+  <si>
+    <t>Adobe-B6</t>
+  </si>
+  <si>
+    <t>Adobe-B8</t>
+  </si>
+  <si>
+    <t>Adobe-C2</t>
+  </si>
+  <si>
+    <t>Briarwood-D9</t>
+  </si>
+  <si>
+    <t>CVID-0825-B1</t>
+  </si>
+  <si>
+    <t>CVID-0825-C10</t>
+  </si>
+  <si>
+    <t>CVID-0911-F4</t>
+  </si>
+  <si>
+    <t>CVID-1006-G6</t>
+  </si>
+  <si>
+    <t>CVID-1006-G7</t>
+  </si>
+  <si>
+    <t>CVID-1006-H2</t>
+  </si>
+  <si>
+    <t>CVID-1006-H3</t>
+  </si>
+  <si>
+    <t>James-A4</t>
+  </si>
+  <si>
+    <t>James-A5</t>
+  </si>
+  <si>
+    <t>ME-F-1</t>
+  </si>
+  <si>
+    <t>ME-F-2</t>
+  </si>
+  <si>
+    <t>ME-F-3</t>
+  </si>
+  <si>
+    <t>ME-F-9</t>
+  </si>
+  <si>
+    <t>ME-M-1</t>
+  </si>
+  <si>
+    <t>ME-M-2</t>
+  </si>
+  <si>
+    <t>ME-M-4</t>
+  </si>
+  <si>
+    <t>ME-M-6</t>
+  </si>
+  <si>
+    <t>ME-M-8</t>
+  </si>
+  <si>
+    <t>ME-M-10</t>
+  </si>
+  <si>
+    <t>ME-M-11</t>
+  </si>
+  <si>
+    <t>ME-M-14</t>
+  </si>
+  <si>
+    <t>ME-M-17</t>
+  </si>
+  <si>
+    <t>ME-M-18</t>
+  </si>
+  <si>
+    <t>ME-M-19</t>
+  </si>
+  <si>
+    <t>ME-M-20</t>
+  </si>
+  <si>
+    <t>Myrtle-D5</t>
+  </si>
+  <si>
+    <t>Myrtle-D11</t>
+  </si>
+  <si>
+    <t>Myrtle-E9</t>
+  </si>
+  <si>
+    <t>OH-M-5</t>
+  </si>
+  <si>
+    <t>Peach-8-F7</t>
+  </si>
+  <si>
+    <t>Peach-9-F8</t>
+  </si>
+  <si>
+    <t>Peach-10-F10</t>
+  </si>
+  <si>
+    <t>Peach-13-H7</t>
+  </si>
+  <si>
+    <t>Penn-F-1</t>
+  </si>
+  <si>
+    <t>Penn-F-2</t>
+  </si>
+  <si>
+    <t>Penn-F-3</t>
+  </si>
+  <si>
+    <t>Penn-F-9</t>
+  </si>
+  <si>
+    <t>Penn-F-12</t>
+  </si>
+  <si>
+    <t>Penn-M-2</t>
+  </si>
+  <si>
+    <t>Penn-M-8</t>
+  </si>
+  <si>
+    <t>Penn-M-10</t>
+  </si>
+  <si>
+    <t>Penn-M-11</t>
+  </si>
+  <si>
+    <t>Penn-M-14</t>
+  </si>
+  <si>
+    <t>Penn-M-15</t>
+  </si>
+  <si>
+    <t>ME-M-3</t>
+  </si>
+  <si>
+    <t>500-F-21</t>
+  </si>
+  <si>
+    <t>ME-M-7</t>
+  </si>
+  <si>
+    <t>Penn-F-4</t>
+  </si>
+  <si>
+    <t>Penn-F-6</t>
   </si>
 </sst>
 </file>
@@ -1762,13 +2065,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64DCA32-379A-8542-91DE-2D3EB11B49A9}">
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:F161"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="6" max="6" width="61.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1784,8 +2088,11 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -1801,8 +2108,11 @@
       <c r="E2" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F2" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1818,8 +2128,11 @@
       <c r="E3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F3" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1835,8 +2148,11 @@
       <c r="E4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1852,8 +2168,11 @@
       <c r="E5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1869,8 +2188,11 @@
       <c r="E6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1886,8 +2208,11 @@
       <c r="E7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>19</v>
       </c>
@@ -1903,8 +2228,11 @@
       <c r="E8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1920,8 +2248,11 @@
       <c r="E9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F9" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1937,8 +2268,11 @@
       <c r="E10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F10" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1954,8 +2288,11 @@
       <c r="E11" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F11" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -1971,8 +2308,11 @@
       <c r="E12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F12" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -1988,8 +2328,11 @@
       <c r="E13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -2005,8 +2348,11 @@
       <c r="E14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F14" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -2022,8 +2368,11 @@
       <c r="E15" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F15" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2039,8 +2388,11 @@
       <c r="E16" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>37</v>
       </c>
@@ -2056,8 +2408,11 @@
       <c r="E17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F17" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2073,8 +2428,11 @@
       <c r="E18" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F18" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -2090,8 +2448,11 @@
       <c r="E19" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -2107,8 +2468,11 @@
       <c r="E20" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F20" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>45</v>
       </c>
@@ -2124,8 +2488,11 @@
       <c r="E21" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F21" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2141,8 +2508,11 @@
       <c r="E22" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F22" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2158,8 +2528,11 @@
       <c r="E23" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F23" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>51</v>
       </c>
@@ -2175,8 +2548,11 @@
       <c r="E24" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F24" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -2192,8 +2568,11 @@
       <c r="E25" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F25" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>55</v>
       </c>
@@ -2209,8 +2588,11 @@
       <c r="E26" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F26" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>57</v>
       </c>
@@ -2226,8 +2608,11 @@
       <c r="E27" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F27" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2243,8 +2628,11 @@
       <c r="E28" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F28" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2260,8 +2648,11 @@
       <c r="E29" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F29" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2277,8 +2668,11 @@
       <c r="E30" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F30" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -2294,8 +2688,11 @@
       <c r="E31" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F31" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -2311,8 +2708,11 @@
       <c r="E32" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F32" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>69</v>
       </c>
@@ -2328,8 +2728,11 @@
       <c r="E33" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F33" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -2345,8 +2748,11 @@
       <c r="E34" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F34" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>73</v>
       </c>
@@ -2362,8 +2768,11 @@
       <c r="E35" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F35" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>75</v>
       </c>
@@ -2379,8 +2788,11 @@
       <c r="E36" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F36" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>77</v>
       </c>
@@ -2396,8 +2808,11 @@
       <c r="E37" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F37" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>79</v>
       </c>
@@ -2413,8 +2828,11 @@
       <c r="E38" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F38" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -2430,8 +2848,11 @@
       <c r="E39" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F39" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>83</v>
       </c>
@@ -2447,8 +2868,11 @@
       <c r="E40" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F40" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>85</v>
       </c>
@@ -2464,8 +2888,11 @@
       <c r="E41" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F41" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>87</v>
       </c>
@@ -2481,8 +2908,11 @@
       <c r="E42" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F42" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>89</v>
       </c>
@@ -2498,8 +2928,11 @@
       <c r="E43" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F43" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>91</v>
       </c>
@@ -2515,8 +2948,11 @@
       <c r="E44" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F44" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -2532,8 +2968,11 @@
       <c r="E45" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F45" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>95</v>
       </c>
@@ -2549,8 +2988,11 @@
       <c r="E46" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F46" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>97</v>
       </c>
@@ -2566,8 +3008,11 @@
       <c r="E47" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F47" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>99</v>
       </c>
@@ -2583,8 +3028,11 @@
       <c r="E48" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F48" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>101</v>
       </c>
@@ -2600,8 +3048,11 @@
       <c r="E49" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F49" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>103</v>
       </c>
@@ -2617,8 +3068,11 @@
       <c r="E50" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F50" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>105</v>
       </c>
@@ -2634,8 +3088,11 @@
       <c r="E51" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F51" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>107</v>
       </c>
@@ -2651,8 +3108,11 @@
       <c r="E52" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F52" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>109</v>
       </c>
@@ -2668,8 +3128,11 @@
       <c r="E53" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F53" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>111</v>
       </c>
@@ -2685,8 +3148,11 @@
       <c r="E54" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F54" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>113</v>
       </c>
@@ -2702,8 +3168,11 @@
       <c r="E55" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F55" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>115</v>
       </c>
@@ -2719,8 +3188,11 @@
       <c r="E56" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F56" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>117</v>
       </c>
@@ -2736,8 +3208,11 @@
       <c r="E57" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F57" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>119</v>
       </c>
@@ -2753,8 +3228,11 @@
       <c r="E58" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F58" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>121</v>
       </c>
@@ -2770,8 +3248,11 @@
       <c r="E59" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F59" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>123</v>
       </c>
@@ -2787,8 +3268,11 @@
       <c r="E60" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F60" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>125</v>
       </c>
@@ -2804,8 +3288,11 @@
       <c r="E61" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F61" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>127</v>
       </c>
@@ -2821,8 +3308,11 @@
       <c r="E62" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F62" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>129</v>
       </c>
@@ -2838,8 +3328,11 @@
       <c r="E63" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F63" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>131</v>
       </c>
@@ -2855,8 +3348,11 @@
       <c r="E64" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F64" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>134</v>
       </c>
@@ -2872,8 +3368,11 @@
       <c r="E65" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F65" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>136</v>
       </c>
@@ -2889,8 +3388,11 @@
       <c r="E66" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F66" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>138</v>
       </c>
@@ -2906,8 +3408,11 @@
       <c r="E67" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F67" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>140</v>
       </c>
@@ -2923,8 +3428,11 @@
       <c r="E68" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F68" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>142</v>
       </c>
@@ -2940,8 +3448,11 @@
       <c r="E69" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F69" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>144</v>
       </c>
@@ -2957,8 +3468,11 @@
       <c r="E70" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F70" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>146</v>
       </c>
@@ -2974,8 +3488,11 @@
       <c r="E71" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F71" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>148</v>
       </c>
@@ -2991,8 +3508,11 @@
       <c r="E72" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F72" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>150</v>
       </c>
@@ -3008,8 +3528,11 @@
       <c r="E73" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F73" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>152</v>
       </c>
@@ -3025,8 +3548,11 @@
       <c r="E74" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F74" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -3042,8 +3568,11 @@
       <c r="E75" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F75" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>156</v>
       </c>
@@ -3059,8 +3588,11 @@
       <c r="E76" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F76" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>158</v>
       </c>
@@ -3076,8 +3608,11 @@
       <c r="E77" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F77" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>160</v>
       </c>
@@ -3093,8 +3628,11 @@
       <c r="E78" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F78" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>162</v>
       </c>
@@ -3110,8 +3648,11 @@
       <c r="E79" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F79" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>164</v>
       </c>
@@ -3127,8 +3668,11 @@
       <c r="E80" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F80" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>166</v>
       </c>
@@ -3144,8 +3688,11 @@
       <c r="E81" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F81" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>168</v>
       </c>
@@ -3161,8 +3708,11 @@
       <c r="E82" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F82" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>170</v>
       </c>
@@ -3178,8 +3728,11 @@
       <c r="E83" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F83" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>172</v>
       </c>
@@ -3195,8 +3748,11 @@
       <c r="E84" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F84" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>174</v>
       </c>
@@ -3212,8 +3768,11 @@
       <c r="E85" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F85" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>177</v>
       </c>
@@ -3229,8 +3788,11 @@
       <c r="E86" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F86" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>179</v>
       </c>
@@ -3246,8 +3808,11 @@
       <c r="E87" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F87" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>181</v>
       </c>
@@ -3263,8 +3828,11 @@
       <c r="E88" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F88" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>183</v>
       </c>
@@ -3280,8 +3848,11 @@
       <c r="E89" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F89" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>185</v>
       </c>
@@ -3297,8 +3868,11 @@
       <c r="E90" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F90" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>188</v>
       </c>
@@ -3314,8 +3888,11 @@
       <c r="E91" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F91" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>190</v>
       </c>
@@ -3331,8 +3908,11 @@
       <c r="E92" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F92" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>192</v>
       </c>
@@ -3348,8 +3928,11 @@
       <c r="E93" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F93" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>194</v>
       </c>
@@ -3365,8 +3948,11 @@
       <c r="E94" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F94" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>196</v>
       </c>
@@ -3382,8 +3968,11 @@
       <c r="E95" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F95" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>198</v>
       </c>
@@ -3399,8 +3988,11 @@
       <c r="E96" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F96" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>200</v>
       </c>
@@ -3416,8 +4008,11 @@
       <c r="E97" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F97" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>202</v>
       </c>
@@ -3433,8 +4028,11 @@
       <c r="E98" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F98" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>204</v>
       </c>
@@ -3450,8 +4048,11 @@
       <c r="E99" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F99" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>206</v>
       </c>
@@ -3467,8 +4068,11 @@
       <c r="E100" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F100" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>208</v>
       </c>
@@ -3484,8 +4088,11 @@
       <c r="E101" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F101" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>210</v>
       </c>
@@ -3501,8 +4108,11 @@
       <c r="E102" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F102" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>212</v>
       </c>
@@ -3518,8 +4128,11 @@
       <c r="E103" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F103" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>214</v>
       </c>
@@ -3535,8 +4148,11 @@
       <c r="E104" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F104" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>216</v>
       </c>
@@ -3552,8 +4168,11 @@
       <c r="E105" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F105" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B106" t="s">
         <v>219</v>
       </c>
@@ -3567,7 +4186,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B107" t="s">
         <v>221</v>
       </c>
@@ -3581,7 +4200,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B108" t="s">
         <v>222</v>
       </c>
@@ -3595,7 +4214,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B109" t="s">
         <v>223</v>
       </c>
@@ -3609,7 +4228,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B110" t="s">
         <v>224</v>
       </c>
@@ -3623,7 +4242,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B111" t="s">
         <v>225</v>
       </c>
@@ -3637,7 +4256,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B112" t="s">
         <v>226</v>
       </c>

</xml_diff>